<commit_message>
Apply Red and Yellow brand palette to deliverables
</commit_message>
<xml_diff>
--- a/reporting/RedAndYellow_Analytics.xlsx
+++ b/reporting/RedAndYellow_Analytics.xlsx
@@ -31,7 +31,7 @@
     <t>CRM &amp; Academic Analytics - marketing spend through to student outcomes</t>
   </si>
   <si>
-    <t>Generated 09 September 2026 from the dbt warehouse. Catalogue is real; all people and campaigns are synthetic.</t>
+    <t>Generated 10 September 2026 from the dbt warehouse. Catalogue is real; all people and campaigns are synthetic.</t>
   </si>
   <si>
     <t>1,500,000</t>
@@ -250,13 +250,13 @@
     <t>Postgraduate Diploma in Digital Marketing</t>
   </si>
   <si>
+    <t>Data Analysis</t>
+  </si>
+  <si>
     <t>Strategic Foresight for Leaders</t>
   </si>
   <si>
     <t>Executive education</t>
-  </si>
-  <si>
-    <t>Data Analysis</t>
   </si>
   <si>
     <t>Sports Sponsorship Marketing</t>
@@ -4009,14 +4009,14 @@
     <font>
       <b/>
       <sz val="22"/>
-      <color rgb="FF22252A"/>
+      <color rgb="FF1D1D1B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF5A6472"/>
+      <color rgb="FF60646B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4024,14 +4024,14 @@
     <font>
       <b/>
       <sz val="26"/>
-      <color rgb="FFE03127"/>
+      <color rgb="FFF52635"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF5A6472"/>
+      <color rgb="FF60646B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4039,7 +4039,7 @@
     <font>
       <b/>
       <sz val="13"/>
-      <color rgb="FF22252A"/>
+      <color rgb="FFF52635"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4055,20 +4055,20 @@
     <font>
       <i/>
       <sz val="10"/>
-      <color rgb="FF5A6472"/>
+      <color rgb="FF60646B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF22252A"/>
+      <color rgb="FF1D1D1B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4077,13 +4077,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF22252A"/>
+        <fgColor rgb="FF1D1D1B"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF6D6"/>
+        <fgColor rgb="FFFFF9F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4100,23 +4106,23 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color rgb="FFD8DDE4"/>
+      <bottom style="medium">
+        <color rgb="FFFFB71B"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF22252A"/>
+        <color rgb="FF1D1D1B"/>
       </left>
       <right style="thin">
-        <color rgb="FF22252A"/>
+        <color rgb="FF1D1D1B"/>
       </right>
       <top style="thin">
-        <color rgb="FF22252A"/>
+        <color rgb="FF1D1D1B"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF22252A"/>
+        <color rgb="FF1D1D1B"/>
       </bottom>
       <diagonal/>
     </border>
@@ -4137,16 +4143,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFFFC629"/>
+        <color rgb="FFFFB71B"/>
       </left>
       <right style="thin">
-        <color rgb="FFFFC629"/>
+        <color rgb="FFFFB71B"/>
       </right>
       <top style="thin">
-        <color rgb="FFFFC629"/>
+        <color rgb="FFFFB71B"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFFFC629"/>
+        <color rgb="FFFFB71B"/>
       </bottom>
       <diagonal/>
     </border>
@@ -4170,13 +4176,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4247,7 +4253,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="E03127"/>
+              <a:srgbClr val="F52635"/>
             </a:solidFill>
           </c:spPr>
           <c:cat>
@@ -4374,7 +4380,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="2E6E8E"/>
+              <a:srgbClr val="007C83"/>
             </a:solidFill>
           </c:spPr>
           <c:cat>
@@ -4537,7 +4543,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="4C9F70"/>
+              <a:srgbClr val="008C45"/>
             </a:solidFill>
           </c:spPr>
           <c:cat>
@@ -4700,7 +4706,7 @@
           <c:spPr>
             <a:ln w="28575">
               <a:solidFill>
-                <a:srgbClr val="E03127"/>
+                <a:srgbClr val="F52635"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -4849,7 +4855,7 @@
           <c:spPr>
             <a:ln w="28575">
               <a:solidFill>
-                <a:srgbClr val="F0A202"/>
+                <a:srgbClr val="E39B16"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -5088,7 +5094,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="C7522A"/>
+              <a:srgbClr val="D9574A"/>
             </a:solidFill>
           </c:spPr>
           <c:cat>
@@ -6976,51 +6982,51 @@
         <v>75</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>55</v>
       </c>
       <c r="E26" s="10">
-        <v>27000</v>
+        <v>13500</v>
       </c>
       <c r="F26" s="8">
-        <v>15963</v>
+        <v>15801</v>
       </c>
       <c r="G26" s="8">
         <v>6474</v>
       </c>
       <c r="H26" s="12">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="I26" s="10">
-        <v>143879154</v>
+        <v>71780786</v>
       </c>
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>77</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>54</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>55</v>
       </c>
       <c r="E27" s="10">
-        <v>13500</v>
+        <v>27000</v>
       </c>
       <c r="F27" s="8">
-        <v>15801</v>
+        <v>15963</v>
       </c>
       <c r="G27" s="8">
         <v>6474</v>
       </c>
       <c r="H27" s="12">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="I27" s="10">
-        <v>71780786</v>
+        <v>143879154</v>
       </c>
     </row>
     <row r="28" spans="2:9">
@@ -14723,7 +14729,7 @@
         <v>1243</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>55</v>
@@ -15275,7 +15281,7 @@
         <v>1267</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>55</v>
@@ -15446,7 +15452,7 @@
     </row>
     <row r="34" spans="2:10">
       <c r="B34" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>54</v>
@@ -16094,7 +16100,7 @@
         <v>1282</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>55</v>
@@ -16791,7 +16797,7 @@
         <v>1297</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D82" s="7" t="s">
         <v>55</v>
@@ -17045,10 +17051,10 @@
     </row>
     <row r="91" spans="2:10">
       <c r="B91" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D91" s="7" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Refine KPI presentation across Power BI and Excel
</commit_message>
<xml_diff>
--- a/reporting/RedAndYellow_Analytics.xlsx
+++ b/reporting/RedAndYellow_Analytics.xlsx
@@ -199,15 +199,15 @@
     <t>Certificate</t>
   </si>
   <si>
+    <t>Higher Certificate in Marketing and Branding</t>
+  </si>
+  <si>
+    <t>On-campus</t>
+  </si>
+  <si>
     <t>Copywriting</t>
   </si>
   <si>
-    <t>Higher Certificate in Marketing and Branding</t>
-  </si>
-  <si>
-    <t>On-campus</t>
-  </si>
-  <si>
     <t>Project Management</t>
   </si>
   <si>
@@ -244,19 +244,19 @@
     <t>Creative Thinking</t>
   </si>
   <si>
+    <t>Postgraduate Diploma in Digital Marketing</t>
+  </si>
+  <si>
     <t>Digital Content &amp; Copywriting</t>
   </si>
   <si>
-    <t>Postgraduate Diploma in Digital Marketing</t>
+    <t>Strategic Foresight for Leaders</t>
+  </si>
+  <si>
+    <t>Executive education</t>
   </si>
   <si>
     <t>Data Analysis</t>
-  </si>
-  <si>
-    <t>Strategic Foresight for Leaders</t>
-  </si>
-  <si>
-    <t>Executive education</t>
   </si>
   <si>
     <t>Sports Sponsorship Marketing</t>
@@ -4068,12 +4068,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7E3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -4094,12 +4100,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE9C46A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE9C46A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE9C46A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE9C46A"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -4164,56 +4185,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFBFBFC"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color rgb="FFD8DDE4"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD8DDE4"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD8DDE4"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD8DDE4"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -5902,36 +5899,6 @@
     <mergeCell ref="H13:J13"/>
     <mergeCell ref="B24:I26"/>
   </mergeCells>
-  <conditionalFormatting sqref="B11:D13">
-    <cfRule type="notContainsErrors" dxfId="0" priority="4">
-      <formula>NOT(ISERROR(B11))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B7:D9">
-    <cfRule type="notContainsErrors" dxfId="0" priority="1">
-      <formula>NOT(ISERROR(B7))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E11:G13">
-    <cfRule type="notContainsErrors" dxfId="0" priority="5">
-      <formula>NOT(ISERROR(E11))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:G9">
-    <cfRule type="notContainsErrors" dxfId="0" priority="2">
-      <formula>NOT(ISERROR(E7))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H11:J13">
-    <cfRule type="notContainsErrors" dxfId="0" priority="6">
-      <formula>NOT(ISERROR(H11))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7:J9">
-    <cfRule type="notContainsErrors" dxfId="0" priority="3">
-      <formula>NOT(ISERROR(H7))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -6576,46 +6543,46 @@
         <v>58</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="10">
-        <v>13500</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="E9" s="10"/>
       <c r="F9" s="8">
-        <v>15796</v>
+        <v>15818</v>
       </c>
       <c r="G9" s="8">
         <v>6586</v>
       </c>
-      <c r="H9" s="12">
-        <v>14.8</v>
-      </c>
-      <c r="I9" s="10">
-        <v>73640481</v>
-      </c>
+      <c r="H9" s="12"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="2:9">
       <c r="B10" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="10"/>
+        <v>55</v>
+      </c>
+      <c r="E10" s="10">
+        <v>13500</v>
+      </c>
       <c r="F10" s="8">
-        <v>15818</v>
+        <v>15796</v>
       </c>
       <c r="G10" s="8">
         <v>6586</v>
       </c>
-      <c r="H10" s="12"/>
-      <c r="I10" s="10"/>
+      <c r="H10" s="12">
+        <v>14.8</v>
+      </c>
+      <c r="I10" s="10">
+        <v>73640481</v>
+      </c>
     </row>
     <row r="11" spans="2:9">
       <c r="B11" s="7" t="s">
@@ -6645,7 +6612,7 @@
     </row>
     <row r="12" spans="2:9">
       <c r="B12" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>57</v>
@@ -6671,7 +6638,7 @@
         <v>57</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="8">
@@ -6841,7 +6808,7 @@
         <v>65</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E20" s="10"/>
       <c r="F20" s="8">
@@ -6936,97 +6903,97 @@
         <v>73</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E24" s="10">
-        <v>14900</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="E24" s="10"/>
       <c r="F24" s="8">
-        <v>15683</v>
+        <v>15650</v>
       </c>
       <c r="G24" s="8">
         <v>6499</v>
       </c>
-      <c r="H24" s="12">
-        <v>15</v>
-      </c>
-      <c r="I24" s="10">
-        <v>79792859</v>
-      </c>
+      <c r="H24" s="12"/>
+      <c r="I24" s="10"/>
     </row>
     <row r="25" spans="2:9">
       <c r="B25" s="7" t="s">
         <v>74</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="E25" s="10"/>
+        <v>55</v>
+      </c>
+      <c r="E25" s="10">
+        <v>14900</v>
+      </c>
       <c r="F25" s="8">
-        <v>15650</v>
+        <v>15683</v>
       </c>
       <c r="G25" s="8">
         <v>6499</v>
       </c>
-      <c r="H25" s="12"/>
-      <c r="I25" s="10"/>
+      <c r="H25" s="12">
+        <v>15</v>
+      </c>
+      <c r="I25" s="10">
+        <v>79792859</v>
+      </c>
     </row>
     <row r="26" spans="2:9">
       <c r="B26" s="7" t="s">
         <v>75</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>55</v>
       </c>
       <c r="E26" s="10">
-        <v>13500</v>
+        <v>27000</v>
       </c>
       <c r="F26" s="8">
-        <v>15801</v>
+        <v>15963</v>
       </c>
       <c r="G26" s="8">
         <v>6474</v>
       </c>
       <c r="H26" s="12">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="I26" s="10">
-        <v>71780786</v>
+        <v>143879154</v>
       </c>
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>55</v>
       </c>
       <c r="E27" s="10">
-        <v>27000</v>
+        <v>13500</v>
       </c>
       <c r="F27" s="8">
-        <v>15963</v>
+        <v>15801</v>
       </c>
       <c r="G27" s="8">
         <v>6474</v>
       </c>
       <c r="H27" s="12">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="I27" s="10">
-        <v>143879154</v>
+        <v>71780786</v>
       </c>
     </row>
     <row r="28" spans="2:9">
@@ -7215,7 +7182,7 @@
         <v>57</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E36" s="10"/>
       <c r="F36" s="8">
@@ -14729,7 +14696,7 @@
         <v>1243</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>55</v>
@@ -14993,7 +14960,7 @@
         <v>1256</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>1240</v>
@@ -15020,7 +14987,7 @@
         <v>1256</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>1240</v>
@@ -15047,7 +15014,7 @@
         <v>1256</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>1240</v>
@@ -15126,7 +15093,7 @@
         <v>65</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>1240</v>
@@ -15153,7 +15120,7 @@
         <v>1263</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>1240</v>
@@ -15180,7 +15147,7 @@
         <v>1263</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>1240</v>
@@ -15257,7 +15224,7 @@
         <v>1263</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>1240</v>
@@ -15281,7 +15248,7 @@
         <v>1267</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>55</v>
@@ -15336,7 +15303,7 @@
     </row>
     <row r="30" spans="2:10">
       <c r="B30" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>54</v>
@@ -15452,7 +15419,7 @@
     </row>
     <row r="34" spans="2:10">
       <c r="B34" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>54</v>
@@ -15622,7 +15589,7 @@
     </row>
     <row r="40" spans="2:10">
       <c r="B40" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>54</v>
@@ -15829,7 +15796,7 @@
         <v>57</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E47" s="7" t="s">
         <v>1240</v>
@@ -15883,7 +15850,7 @@
         <v>57</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E49" s="7" t="s">
         <v>1240</v>
@@ -15910,7 +15877,7 @@
         <v>57</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E50" s="7" t="s">
         <v>1240</v>
@@ -15931,13 +15898,13 @@
     </row>
     <row r="51" spans="2:10">
       <c r="B51" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>57</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E51" s="7" t="s">
         <v>1240</v>
@@ -15958,7 +15925,7 @@
     </row>
     <row r="52" spans="2:10">
       <c r="B52" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C52" s="7" t="s">
         <v>57</v>
@@ -16018,7 +15985,7 @@
         <v>57</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E54" s="7" t="s">
         <v>1240</v>
@@ -16100,7 +16067,7 @@
         <v>1282</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>55</v>
@@ -16572,13 +16539,13 @@
     </row>
     <row r="74" spans="2:10">
       <c r="B74" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C74" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>1240</v>
@@ -16605,7 +16572,7 @@
         <v>65</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E75" s="7" t="s">
         <v>1240</v>
@@ -16632,7 +16599,7 @@
         <v>65</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E76" s="7" t="s">
         <v>1240</v>
@@ -16797,7 +16764,7 @@
         <v>1297</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D82" s="7" t="s">
         <v>55</v>
@@ -17051,10 +17018,10 @@
     </row>
     <row r="91" spans="2:10">
       <c r="B91" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C91" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="C91" s="7" t="s">
-        <v>77</v>
       </c>
       <c r="D91" s="7" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Clarify GA4 routes and add BigQuery target
</commit_message>
<xml_diff>
--- a/reporting/RedAndYellow_Analytics.xlsx
+++ b/reporting/RedAndYellow_Analytics.xlsx
@@ -248,12 +248,12 @@
     <t>Part-Time Postgraduate Diploma in Management</t>
   </si>
   <si>
+    <t>Creative Thinking</t>
+  </si>
+  <si>
     <t>Design Thinking</t>
   </si>
   <si>
-    <t>Creative Thinking</t>
-  </si>
-  <si>
     <t>People Management</t>
   </si>
   <si>
@@ -3806,10 +3806,10 @@
     <t>Platform</t>
   </si>
   <si>
-    <t>Fabric silver/gold and GA4 remain gated by external execution.</t>
-  </si>
-  <si>
-    <t>Fix T-SQL compatibility, rerun dbt in Fabric, then add GA4 as dated bronze.</t>
+    <t>Fabric silver/gold remains gated by external execution; GA4 can use the Data API without BigQuery or native BigQuery export for raw events.</t>
+  </si>
+  <si>
+    <t>Keep the Data API route for aggregated campaign KPIs; use native BigQuery export for raw events, then run the shared dbt graph on the BigQuery target.</t>
   </si>
   <si>
     <t>Data engineering</t>
@@ -6752,7 +6752,7 @@
     </row>
     <row r="31" spans="2:10">
       <c r="B31" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>54</v>
@@ -6926,7 +6926,7 @@
     </row>
     <row r="37" spans="2:10">
       <c r="B37" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>54</v>
@@ -9579,19 +9579,19 @@
         <v>55</v>
       </c>
       <c r="E23" s="10">
-        <v>13500</v>
+        <v>4900</v>
       </c>
       <c r="F23" s="8">
-        <v>15794</v>
+        <v>15795</v>
       </c>
       <c r="G23" s="8">
         <v>6516</v>
       </c>
       <c r="H23" s="12">
-        <v>15.1</v>
+        <v>15</v>
       </c>
       <c r="I23" s="10">
-        <v>72441283</v>
+        <v>26454867</v>
       </c>
     </row>
     <row r="24" spans="2:9">
@@ -9605,19 +9605,19 @@
         <v>55</v>
       </c>
       <c r="E24" s="10">
-        <v>4900</v>
+        <v>13500</v>
       </c>
       <c r="F24" s="8">
-        <v>15795</v>
+        <v>15794</v>
       </c>
       <c r="G24" s="8">
         <v>6516</v>
       </c>
       <c r="H24" s="12">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="I24" s="10">
-        <v>26454867</v>
+        <v>72441283</v>
       </c>
     </row>
     <row r="25" spans="2:9">
@@ -9648,7 +9648,7 @@
     </row>
     <row r="26" spans="2:9">
       <c r="B26" s="7" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>61</v>
@@ -9658,7 +9658,7 @@
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="8">
-        <v>15855</v>
+        <v>15865</v>
       </c>
       <c r="G26" s="8">
         <v>6507</v>
@@ -9668,7 +9668,7 @@
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="7" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>61</v>
@@ -9678,7 +9678,7 @@
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="8">
-        <v>15865</v>
+        <v>15855</v>
       </c>
       <c r="G27" s="8">
         <v>6507</v>

</xml_diff>